<commit_message>
Retest Mode 4 Golden Path after Lot-mode bug fixes, fresh screenshots
The 3 Lot-mode stone-material bugs documented as known-issues in
TC-E2E-M4-03/09 (delivery routing, phantom negative stock, BOQ
lump-sum price clobbered) are fixed in stone_slab_inventory
(34be05d + 1e09854). Re-ran the full Mode 4 flow live through the
Odoo web UI via Playwright against a fresh fixture (BOQ0026 -> SO
S00109 -> Project 40 -> 3 Down Payment invoices -> Delivery
EG01/OUT/00064) to verify all 3 fixes hold end-to-end, and replaced
every screenshot + figure in the doc with real captures from this
run. TC-03 and TC-09's know-issue callouts are now green "fixed and
re-verified" notes instead of red bug flags.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-test-cases-e2e-mode4.xlsx
+++ b/client-docs/test-cases/emg-o-test-cases-e2e-mode4.xlsx
@@ -691,14 +691,14 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>BOQ0023 — ลูกค้า "ทดสอบ Mode 4 - Boutique Villa"
+          <t>BOQ0026 — ลูกค้า "ทดสอบ Mode 4 Retest - Riverside Condo"
 2 รายการ: Vietnam Limestone - Slab 0.5 ตร.ม. + Dry-Lay 1.5 ตร.ม.
 Preliminaries 5% + Overhead &amp; Profit 10%</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>สถานะ BOQ เปลี่ยนเป็น "Quotation Generated" เกิด Sale Order ใหม่ 1 ใบอัตโนมัติ ดึงทุกรายการ + ค่า Preliminaries/Overhead มาเป็นบรรทัดในใบเสนอราคาให้ครบ — ตัวอย่างจริง: BOQ0023 (รวม 1,380.00 บาท ก่อน VAT) → SO S00102</t>
+          <t>สถานะ BOQ เปลี่ยนเป็น "Quotation Generated" เกิด Sale Order ใหม่ 1 ใบอัตโนมัติ ดึงทุกรายการ + ค่า Preliminaries/Overhead มาเป็นบรรทัดในใบเสนอราคาให้ครบ — ตัวอย่างจริง: BOQ0026 (รวม 1,380.00 บาท ก่อน VAT) → SO S00109</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>บรรทัดผูกกับ Lot ที่เลือกสำเร็จ จำนวนเปลี่ยนเป็น 0.5 ตร.ม. ตามที่กรอก — ตัวอย่างจริง: ราคาต่อหน่วยเปลี่ยนจาก 900.00 เป็น 800.00×0.5 = 400.00 บาท (ดูหมายเหตุด้านซ้าย)</t>
+          <t>บรรทัดผูกกับ Lot ที่เลือกสำเร็จ จำนวนเปลี่ยนเป็น 0.5 ตร.ม. ตามที่กรอก ราคารวมของบรรทัดยังคงเท่าเดิมกับที่ BOQ ตั้งไว้เป๊ะ (ระบบคำนวณราคาต่อหน่วยใหม่ให้เอง) — ตัวอย่างจริง: ราคาต่อหน่วยเปลี่ยนจาก 900.00 (ที่จำนวน 1 หน่วยตั้งต้น) เป็น 1,800.00 บาท/ตร.ม. × 0.5 ตร.ม. = ยอดรวม 900.00 บาท เท่าเดิมทุกบาท</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>🔴 พบปัญหาจริง (ยังไม่แก้): (1) ช่องแสดงสต็อกคงเหลือของ Lot นี้ขึ้นแค่ 0.54 ตร.ม. ทั้งที่ของจริงมี 2.34 ตร.ม. อยู่หน้าคลัง (2) หลังกดยืนยันจำนวนแล้ว ราคาต่อหน่วยของบรรทัดจะเปลี่ยนจากราคาที่ BOQ ตั้งไว้ (900 บาท) เป็นราคาป้ายสินค้าปกติคูณจำนวนใหม่ (400 บาท) โดยไม่มีคำเตือนใดๆ — เป็นบั๊กจริงของระบบ ไม่ใช่ขั้นตอนที่ตั้งใจให้เป็นแบบนี้ ผู้ใช้ควรตรวจราคาทุกครั้งหลังทำขั้นนี้</t>
+          <t>✅ เคยพบปัญหาจริงตรงนี้ (ราคาที่ BOQ ตั้งไว้ถูกเขียนทับด้วยราคาป้ายสินค้าปกติ) — แก้ไขแล้วและทดสอบซ้ำผ่านในรอบนี้: ระบบคำนวณราคาต่อหน่วยใหม่ให้อัตโนมัติจากยอดรวมเดิมที่ BOQ ตั้งไว้ ไม่ใช้ราคาป้ายสินค้าอีกต่อไป</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -934,7 +934,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>SO เปลี่ยนสถานะเป็น "Sales Order" เกิดปุ่ม/สถิติใหม่มุมบน: "Projects 1", "Tasks", "Delivery 1", "Invoices" — ไม่ต้องสร้าง Project เองแยกต่างหาก — ตัวอย่างจริง: S00102 (ยอดรวมหลังปรับราคาจาก TC-03 = 941.60 บาท รวม VAT) → Project id 38</t>
+          <t>SO เปลี่ยนสถานะเป็น "Sales Order" เกิดปุ่ม/สถิติใหม่มุมบน: "Projects 1", "Tasks", "Delivery 1", "Invoices" — ไม่ต้องสร้าง Project เองแยกต่างหาก — ตัวอย่างจริง: S00109 (ยอดรวม 1,476.60 บาท รวม VAT) → Project id 40</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>เห็น Task ครบ 1 งานต่อ 1 บรรทัดสินค้า/บริการ — ตัวอย่างจริง: 4 Tasks ("Vietnam Limestone - Slab...", "Dry-Lay", "BOQ Summary Line Preliminaries (5%)", "BOQ Summary Line Overhead &amp; Profit (10%)")</t>
+          <t>เห็น Task ครบ 1 งานต่อ 1 บรรทัดสินค้า/บริการ — ตัวอย่างจริง: 4 Tasks ("Vietnam Limestone - Slab (ปูพื้นระเบียง)...", "Dry-Lay", "BOQ Summary Line Preliminaries (5%)", "BOQ Summary Line Overhead &amp; Profit (10%)")</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอด 30% ของยอดรวม SO — ตัวอย่างจริง: INV/2026/00012 (282.48 บาท จาก 941.60 × 30%)</t>
+          <t>ใบแจ้งหนี้สถานะ Posted ยอด 30% ของยอดรวม SO — ตัวอย่างจริง: INV/2026/00015 (442.98 บาท จาก 1,476.60 × 30%)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอด 40% ของยอดรวม SO — ตัวอย่างจริง: INV/2026/00013 (376.64 บาท จาก 941.60 × 40%)</t>
+          <t>ใบแจ้งหนี้สถานะ Posted ยอด 40% ของยอดรวม SO — ตัวอย่างจริง: INV/2026/00016 (590.64 บาท จาก 1,476.60 × 40%)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอดงวดสุดท้าย รวม 3 ใบแล้วเท่ากับยอด SO เป๊ะ — ตัวอย่างจริง: INV/2026/00014 (282.48 บาท) รวม 3 ใบ = 282.48 + 376.64 + 282.48 = 941.60 บาท ตรงกับยอด SO พอดี</t>
+          <t>ใบแจ้งหนี้สถานะ Posted ยอดงวดสุดท้าย รวม 3 ใบแล้วเท่ากับยอด SO เป๊ะ — ตัวอย่างจริง: INV/2026/00017 (442.98 บาท) รวม 3 ใบ = 442.98 + 590.64 + 442.98 = 1,476.60 บาท ตรงกับยอด SO พอดี</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบส่งของเปลี่ยนสถานะเป็น Done — ตัวอย่างจริง: EG01/OUT/00059 (Vietnam Limestone - Slab 0.5 ตร.ม.)</t>
+          <t>ใบส่งของเปลี่ยนสถานะเป็น Done ดึงสต็อกจากจุดที่ของจริงอยู่ถูกต้อง — ตัวอย่างจริง: EG01/OUT/00064 (Vietnam Limestone - Slab 0.5 ตร.ม., Pick From "Stone Inventory/Stone Available")</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>🔴 พบปัญหาจริง (ยังไม่แก้): ระบบดึงสต็อกจากจุดพัก "Stone Hold" เสมอสำหรับสินค้าโหมด Lot ทั้งที่โหมดนี้ไม่เคยมีขั้นตอนย้ายของจริงไปที่จุดพักนั้นเลย (ต่างจาก Serial/Cut-to-Order) ผลคือยอดคงเหลือที่จุดพักนั้นติดลบเพิ่มขึ้นเรื่อยๆ ทุกครั้งที่ส่งของ (จาก -1.8 เป็น -2.3 ตร.ม.ในรอบนี้) แม้ของจริงจะยังอยู่ครบที่หน้าคลัง — ใบส่งของยังคง Validate ผ่านได้ตามปกติ ไม่กระทบขั้นตอนที่ผู้ใช้เห็น</t>
+          <t>✅ เคยพบปัญหาจริงตรงนี้ (ระบบดึงสต็อกจากจุดพัก "Stone Hold" ที่โหมด Lot ไม่เคยย้ายของเข้าจริง ทำให้ยอดติดลบเพิ่มขึ้นทุกครั้งที่ส่งของ) — แก้ไขแล้วและทดสอบซ้ำผ่านในรอบนี้: ระบบดึงสต็อกจากจุดที่ของจริงอยู่ ("Stone Available") แทน ดูรายละเอียดที่ปุ่ม "Details" ในรายการส่งของ</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -1506,7 +1506,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Task ขึ้นเครื่องหมายเสร็จ และ Milestone ที่ผูกกับ Task นั้นเปลี่ยนเป็น "Reached" ให้อัตโนมัติ โดยไม่ต้องไปกดยืนยัน Milestone แยกต่างหาก — ตัวอย่างจริง: Milestone "ปูพื้นหินเสร็จสมบูรณ์ (Dry-Lay Complete)" ขึ้นเครื่องหมายถูกในหน้า Project Dashboard ทันที</t>
+          <t>Task ขึ้นเครื่องหมายเสร็จ และ Milestone ที่ผูกกับ Task นั้นเปลี่ยนเป็น "Reached" ให้อัตโนมัติ โดยไม่ต้องไปกดยืนยัน Milestone แยกต่างหาก — ตัวอย่างจริง: Milestone "ปูพื้นระเบียงเสร็จสมบูรณ์ (Dry-Lay Complete)" ขึ้นเครื่องหมายถูกในหน้า Project Dashboard ทันที</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>เห็นยอดรายได้แยกตามหมวด (Materials / Other Services / Down Payments) รวมกันแล้วต้องเท่ากับยอดใบแจ้งหนี้ทั้งหมด (ไม่รวม VAT) — ตัวอย่างจริง: Other Services 480 + Materials 400 = Total Revenues 880 บาท ตรงกับยอด Invoiced 880 บาททั้งหมด (ออกครบ 3 งวดแล้ว จึง Expected = Invoiced พอดี ไม่มียอดค้าง "To Invoice")</t>
+          <t>เห็นยอดรายได้แยกตามหมวด (Materials / Other Services / Down Payments) รวมกันแล้วต้องเท่ากับยอดใบแจ้งหนี้ทั้งหมด (ไม่รวม VAT) — ตัวอย่างจริง: Other Services 480 + Materials 900 = Total Revenues 1,380 บาท ตรงกับยอด Invoiced 1,380 บาททั้งหมด (ออกครบ 3 งวดแล้ว จึง Expected = Invoiced พอดี ไม่มียอดค้าง "To Invoice" — ยอด Materials 900 นี้คือหลักฐานว่าราคาที่ BOQ ตั้งไว้ไม่ถูกเขียนทับแล้ว, ดู TC-03)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>เดบิต/เครดิตสมดุลกัน (รวมเท่ากันทั้ง 2 ฝั่ง) เห็น Analytic Distribution ผูกกับบัญชี Analytic ของโปรเจกต์นี้บนบรรทัดรายได้ — ตัวอย่างจริง: INV/2026/00014 เดบิต Trade Receivables 282.48 = เครดิต Down Payment 264.00 + Output VAT 18.48 พอดี พร้อมป้าย Analytic "BOQ0023 - ทดสอบ Mode 4..."</t>
+          <t>เดบิต/เครดิตสมดุลกัน (รวมเท่ากันทั้ง 2 ฝั่ง) เห็น Analytic Distribution ผูกกับบัญชี Analytic ของโปรเจกต์นี้บนบรรทัดรายได้ — ตัวอย่างจริง: INV/2026/00017 เดบิต Trade Receivables 442.98 = เครดิต Down Payment 414.00 + Output VAT 28.98 พอดี พร้อมป้าย Analytic "BOQ0026 - ทดสอบ Mode 4 Retest..."</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">

</xml_diff>